<commit_message>
Fixed timesheet hour and salary issue. add itemname2 in item save api. add bankdate parameter in payroll_insert sp
</commit_message>
<xml_diff>
--- a/KLS.API/wwwroot/Payroll/Tax Import.xlsx
+++ b/KLS.API/wwwroot/Payroll/Tax Import.xlsx
@@ -1,31 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\DO NOT DELETE - WORK BKP\IMPORT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7385D3A-1979-4322-A154-43D05ACBA6F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A45C876-4901-45F0-9D99-09B98C0B57B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$21</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Payment Date</t>
   </si>
@@ -40,14 +52,82 @@
   </si>
   <si>
     <t>BankDate</t>
+  </si>
+  <si>
+    <t>06/13/2025</t>
+  </si>
+  <si>
+    <t>06/20/2025</t>
+  </si>
+  <si>
+    <t>06/27/2025</t>
+  </si>
+  <si>
+    <t>07/03/2025</t>
+  </si>
+  <si>
+    <t>07/11/2025</t>
+  </si>
+  <si>
+    <t>07/18/2025</t>
+  </si>
+  <si>
+    <t>07/25/2025</t>
+  </si>
+  <si>
+    <t>08/01/2025</t>
+  </si>
+  <si>
+    <t>08/08/2025</t>
+  </si>
+  <si>
+    <t>08/15/2025</t>
+  </si>
+  <si>
+    <t>08/22/2025</t>
+  </si>
+  <si>
+    <t>08/29/2025</t>
+  </si>
+  <si>
+    <t>09/05/2025</t>
+  </si>
+  <si>
+    <t>09/12/2025</t>
+  </si>
+  <si>
+    <t>10/03/2025</t>
+  </si>
+  <si>
+    <t>09/19/2025</t>
+  </si>
+  <si>
+    <t>09/26/2025</t>
+  </si>
+  <si>
+    <t>10/10/2025</t>
+  </si>
+  <si>
+    <t>10/17/2025</t>
+  </si>
+  <si>
+    <t>10/24/2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -75,9 +155,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -358,69 +440,251 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5546875" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
-        <v>45274</v>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="B2">
-        <v>-3200.99</v>
+        <v>195.34</v>
       </c>
       <c r="E2" s="1">
-        <v>45275</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
-        <v>45275</v>
+        <v>45820</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="B3">
-        <v>-3662.65</v>
+        <v>195.34</v>
       </c>
       <c r="E3" s="1">
-        <v>45276</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <v>45281</v>
+        <v>45828</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="B4">
-        <v>-3361.39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>45286</v>
+        <v>195.34</v>
+      </c>
+      <c r="E4" s="1">
+        <v>45834</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
       </c>
       <c r="B5">
-        <v>-2121.19</v>
+        <v>195.34</v>
+      </c>
+      <c r="E5" s="1">
+        <v>45841</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>195.34</v>
+      </c>
+      <c r="E6" s="1">
+        <v>45848</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>195.34</v>
+      </c>
+      <c r="E7" s="1">
+        <v>45855</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8">
+        <v>195.34</v>
+      </c>
+      <c r="E8" s="1">
+        <v>45862</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <v>195.34</v>
+      </c>
+      <c r="E9" s="1">
+        <v>45869</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10">
+        <v>195.34</v>
+      </c>
+      <c r="E10" s="1">
+        <v>45876</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11">
+        <v>195.34</v>
+      </c>
+      <c r="E11" s="1">
+        <v>45883</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12">
+        <v>195.34</v>
+      </c>
+      <c r="E12" s="1">
+        <v>45890</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13">
+        <v>195.34</v>
+      </c>
+      <c r="E13" s="1">
+        <v>45897</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14">
+        <v>195.34</v>
+      </c>
+      <c r="E14" s="1">
+        <v>45904</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15">
+        <v>195.34</v>
+      </c>
+      <c r="E15" s="1">
+        <v>45911</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16">
+        <v>195.34</v>
+      </c>
+      <c r="E16" s="1">
+        <v>45918</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17">
+        <v>195.34</v>
+      </c>
+      <c r="E17" s="1">
+        <v>45925</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18">
+        <v>195.34</v>
+      </c>
+      <c r="E18" s="1">
+        <v>45932</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19">
+        <v>195.34</v>
+      </c>
+      <c r="E19" s="1">
+        <v>45939</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20">
+        <v>195.34</v>
+      </c>
+      <c r="E20" s="1">
+        <v>45946</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21">
+        <v>195.34</v>
+      </c>
+      <c r="E21" s="1">
+        <v>45953</v>
       </c>
     </row>
   </sheetData>

</xml_diff>